<commit_message>
Add comprehensive 4-in-1 test suite & security assessment with 300+ test cases per suite, Excel generators, and GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/security-review-latest.xlsx
+++ b/Vulnerability Test Results/security-review-latest.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="502">
   <si>
-    <t>🛡️ MEDICATE — SECURITY FINDINGS REPORT   |   Build #0   |   2026-08-11 16:59:06 UTC</t>
+    <t>🛡️ MEDICATE — SECURITY FINDINGS REPORT   |   Build #0   |   2026-10-27 15:30:28 UTC</t>
   </si>
   <si>
     <t>🔴 Critical: 3</t>
@@ -1363,7 +1363,7 @@
     <t>Scan Date</t>
   </si>
   <si>
-    <t>2026-08-11 16:59:06 UTC</t>
+    <t>2026-10-27 15:30:28 UTC</t>
   </si>
   <si>
     <t>Scanned By</t>

</xml_diff>